<commit_message>
Fixed bug with requests, updated Reuquests with a RESET buttong
</commit_message>
<xml_diff>
--- a/cadet_data/CadetData_Blues.xlsx
+++ b/cadet_data/CadetData_Blues.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94a1dad5ec87e9ff/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94a1dad5ec87e9ff/Documents/Programming/A4Uniforms/cadet_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF3FAB2C-FFCA-45F7-8FDD-EAC7242CA861}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{CF3FAB2C-FFCA-45F7-8FDD-EAC7242CA861}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74397ED7-A490-4DD8-AE34-4ED98ACB2A3A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{03D6A893-5027-493D-A8C5-6DB356B5A452}"/>
   </bookViews>
@@ -83,81 +83,6 @@
     <t>Gender</t>
   </si>
   <si>
-    <t>Short Sleeve Shirt(M/F) -Size</t>
-  </si>
-  <si>
-    <t>Short Sleeve Shirt(M/F) - Qty</t>
-  </si>
-  <si>
-    <t>Long Sleeve Shirt(M/F)  - Size</t>
-  </si>
-  <si>
-    <t>Long Sleeve Shirt(M/F) - Qty</t>
-  </si>
-  <si>
-    <t>Pants (M/F) - Size</t>
-  </si>
-  <si>
-    <t>Pant (M/F) - Qty</t>
-  </si>
-  <si>
-    <t>Service Coat (M/F) - Size</t>
-  </si>
-  <si>
-    <t>Service Coat (M/F0 - Qty</t>
-  </si>
-  <si>
-    <t>Flight Cap (M/F) - Size</t>
-  </si>
-  <si>
-    <t>Flight Cap (M/F) -Qty</t>
-  </si>
-  <si>
-    <t>Lightweight Jacket (M/F) - Size</t>
-  </si>
-  <si>
-    <t>Lightweight Jacket (M/F) - Qty</t>
-  </si>
-  <si>
-    <t>Shoes (M/F) - Size</t>
-  </si>
-  <si>
-    <t>Shoes (M/F) -Qty</t>
-  </si>
-  <si>
-    <t>Pumps (F) - Size</t>
-  </si>
-  <si>
-    <t>Pumps (F) - Qty</t>
-  </si>
-  <si>
-    <t>Skirt (F) - Size</t>
-  </si>
-  <si>
-    <t>Skirt (F) - Qty</t>
-  </si>
-  <si>
-    <t>Neck Tab (F) - Qty</t>
-  </si>
-  <si>
-    <t>Tie(M) - Qty</t>
-  </si>
-  <si>
-    <t>Soft Rank (M/F) - Qty</t>
-  </si>
-  <si>
-    <t>Unisex Socks - Qty</t>
-  </si>
-  <si>
-    <t>Belt - Qty</t>
-  </si>
-  <si>
-    <t>Buckles - Qty</t>
-  </si>
-  <si>
-    <t>Allen, Michael</t>
-  </si>
-  <si>
     <t>AS100</t>
   </si>
   <si>
@@ -167,108 +92,21 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>Calderon, Mia</t>
-  </si>
-  <si>
     <t>F</t>
   </si>
   <si>
-    <t>Emmons, Mckenzie</t>
-  </si>
-  <si>
-    <t>Guttman, Ryan</t>
-  </si>
-  <si>
-    <t>Kieselowsky, Sofiya</t>
-  </si>
-  <si>
-    <t>Krenk, Spencer</t>
-  </si>
-  <si>
     <t>AS150</t>
   </si>
   <si>
-    <t>Roy, Ritika</t>
-  </si>
-  <si>
-    <t>Spurlock, Liam</t>
-  </si>
-  <si>
-    <t>Tsoi, Thomas</t>
-  </si>
-  <si>
-    <t>Anand, Hrishikesh</t>
-  </si>
-  <si>
     <t>AS200</t>
   </si>
   <si>
-    <t>Ben-Zvi, Ari</t>
-  </si>
-  <si>
-    <t>Besana, Anastasia</t>
-  </si>
-  <si>
-    <t>Chung, Ethan</t>
-  </si>
-  <si>
-    <t>Elnasser, Zaid</t>
-  </si>
-  <si>
-    <t>Gentile, Nicholas</t>
-  </si>
-  <si>
-    <t>Gerst, Tyler</t>
-  </si>
-  <si>
     <t>AS250</t>
   </si>
   <si>
-    <t>Gopalakrishnan, Laya</t>
-  </si>
-  <si>
-    <t>Harold, Danille</t>
-  </si>
-  <si>
     <t>AS500</t>
   </si>
   <si>
-    <t>Kelly, Connor</t>
-  </si>
-  <si>
-    <t>Maria, Antonio</t>
-  </si>
-  <si>
-    <t>McCarthy, Norah</t>
-  </si>
-  <si>
-    <t>Miller, Kenneth</t>
-  </si>
-  <si>
-    <t>Nacanaynay, Jakob</t>
-  </si>
-  <si>
-    <t>Park, Jekemiah</t>
-  </si>
-  <si>
-    <t>Racette, Nicholas</t>
-  </si>
-  <si>
-    <t>Smiley, Samuel</t>
-  </si>
-  <si>
-    <t>Sokolowski, James</t>
-  </si>
-  <si>
-    <t>Tama, Charlotte</t>
-  </si>
-  <si>
-    <t>Yap, Nicholas</t>
-  </si>
-  <si>
-    <t>14.5 X 30</t>
-  </si>
-  <si>
     <t>32R</t>
   </si>
   <si>
@@ -278,144 +116,63 @@
     <t>???</t>
   </si>
   <si>
-    <t>Chaney, Jack</t>
-  </si>
-  <si>
     <t>AS300</t>
   </si>
   <si>
-    <t>Chung, Hanna</t>
-  </si>
-  <si>
     <t>6MS</t>
   </si>
   <si>
     <t>10S</t>
   </si>
   <si>
-    <t>Fujimoto, Andrew</t>
-  </si>
-  <si>
     <t>36R</t>
   </si>
   <si>
-    <t>Marino, Frank</t>
-  </si>
-  <si>
-    <t>Martini, Marco</t>
-  </si>
-  <si>
     <t>42L</t>
   </si>
   <si>
-    <t>Martins, Anket</t>
-  </si>
-  <si>
-    <t>McBride, Lindsey</t>
-  </si>
-  <si>
     <t>12R</t>
   </si>
   <si>
-    <t>Melton, Dawson</t>
-  </si>
-  <si>
-    <t>Rahman, Nadia</t>
-  </si>
-  <si>
     <t>W10M</t>
   </si>
   <si>
-    <t>Randall, Conrad</t>
-  </si>
-  <si>
     <t>36S</t>
   </si>
   <si>
-    <t>Shegogue, Thomas</t>
-  </si>
-  <si>
-    <t>Stallone, Thomas</t>
-  </si>
-  <si>
-    <t>Viani, Jared</t>
-  </si>
-  <si>
-    <t>Zegunia, Julia</t>
-  </si>
-  <si>
     <t>8MR</t>
   </si>
   <si>
     <t>M4R</t>
   </si>
   <si>
-    <t>Annor, Reginald</t>
-  </si>
-  <si>
     <t>AS400</t>
   </si>
   <si>
     <t>38L</t>
   </si>
   <si>
-    <t>Chilukuri, Sathya</t>
-  </si>
-  <si>
-    <t>Ettinger, Sophie</t>
-  </si>
-  <si>
     <t>6L</t>
   </si>
   <si>
-    <t>Fancher, Phillip</t>
-  </si>
-  <si>
-    <t>Hunt, Elyse</t>
-  </si>
-  <si>
-    <t>Isaac, Charles</t>
-  </si>
-  <si>
     <t>33R</t>
   </si>
   <si>
-    <t>Kim, Leo</t>
-  </si>
-  <si>
-    <t>Long, John</t>
-  </si>
-  <si>
     <t>44R</t>
   </si>
   <si>
-    <t>Perez, Rodrigo</t>
-  </si>
-  <si>
     <t>42R</t>
   </si>
   <si>
     <t>9.5R</t>
   </si>
   <si>
-    <t>Scalfani-Cohen, Andrew</t>
-  </si>
-  <si>
     <t>40R</t>
   </si>
   <si>
     <t>38R</t>
   </si>
   <si>
-    <t>Szymanski, Zoe</t>
-  </si>
-  <si>
-    <t>Teague, Katie</t>
-  </si>
-  <si>
-    <t>Tremel, Pulani</t>
-  </si>
-  <si>
     <t>4R</t>
   </si>
   <si>
@@ -423,13 +180,256 @@
   </si>
   <si>
     <t>Missing</t>
+  </si>
+  <si>
+    <t>Tie(M)Qty</t>
+  </si>
+  <si>
+    <t>BeltQty</t>
+  </si>
+  <si>
+    <t>BucklesQty</t>
+  </si>
+  <si>
+    <t>ShortSleeveShirt(M/F)Size</t>
+  </si>
+  <si>
+    <t>ShortSleeveShirt(M/F)Qty</t>
+  </si>
+  <si>
+    <t>LongSleeveShirt(M/F)Size</t>
+  </si>
+  <si>
+    <t>LongSleeveShirt(M/F)Qty</t>
+  </si>
+  <si>
+    <t>Pants(M/F)Size</t>
+  </si>
+  <si>
+    <t>Pant(M/F)Qty</t>
+  </si>
+  <si>
+    <t>ServiceCoat(M/F)Size</t>
+  </si>
+  <si>
+    <t>ServiceCoat(M/F0Qty</t>
+  </si>
+  <si>
+    <t>FlightCap(M/F)Size</t>
+  </si>
+  <si>
+    <t>FlightCap(M/F)-Qty</t>
+  </si>
+  <si>
+    <t>LightweightJacket(M/F)Size</t>
+  </si>
+  <si>
+    <t>LightweightJacket(M/F)Qty</t>
+  </si>
+  <si>
+    <t>Shoes(M/F)Size</t>
+  </si>
+  <si>
+    <t>Shoes(M/F)-Qty</t>
+  </si>
+  <si>
+    <t>Pumps(F)Size</t>
+  </si>
+  <si>
+    <t>Pumps(F)Qty</t>
+  </si>
+  <si>
+    <t>Skirt(F)Size</t>
+  </si>
+  <si>
+    <t>Skirt(F)Qty</t>
+  </si>
+  <si>
+    <t>NeckTab(F)Qty</t>
+  </si>
+  <si>
+    <t>SoftRank(M/F)Qty</t>
+  </si>
+  <si>
+    <t>UnisexSocksQty</t>
+  </si>
+  <si>
+    <t>Allen,Michael</t>
+  </si>
+  <si>
+    <t>Calderon,Mia</t>
+  </si>
+  <si>
+    <t>Emmons,Mckenzie</t>
+  </si>
+  <si>
+    <t>Guttman,Ryan</t>
+  </si>
+  <si>
+    <t>Kieselowsky,Sofiya</t>
+  </si>
+  <si>
+    <t>Krenk,Spencer</t>
+  </si>
+  <si>
+    <t>Roy,Ritika</t>
+  </si>
+  <si>
+    <t>Spurlock,Liam</t>
+  </si>
+  <si>
+    <t>Tsoi,Thomas</t>
+  </si>
+  <si>
+    <t>Anand,Hrishikesh</t>
+  </si>
+  <si>
+    <t>Ben-Zvi,Ari</t>
+  </si>
+  <si>
+    <t>Besana,Anastasia</t>
+  </si>
+  <si>
+    <t>Chung,Ethan</t>
+  </si>
+  <si>
+    <t>Elnasser,Zaid</t>
+  </si>
+  <si>
+    <t>Gentile,Nicholas</t>
+  </si>
+  <si>
+    <t>Gerst,Tyler</t>
+  </si>
+  <si>
+    <t>Gopalakrishnan,Laya</t>
+  </si>
+  <si>
+    <t>Harold,Danille</t>
+  </si>
+  <si>
+    <t>Kelly,Connor</t>
+  </si>
+  <si>
+    <t>Maria,Antonio</t>
+  </si>
+  <si>
+    <t>McCarthy,Norah</t>
+  </si>
+  <si>
+    <t>Miller,Kenneth</t>
+  </si>
+  <si>
+    <t>Nacanaynay,Jakob</t>
+  </si>
+  <si>
+    <t>Park,Jekemiah</t>
+  </si>
+  <si>
+    <t>Racette,Nicholas</t>
+  </si>
+  <si>
+    <t>Smiley,Samuel</t>
+  </si>
+  <si>
+    <t>Sokolowski,James</t>
+  </si>
+  <si>
+    <t>Tama,Charlotte</t>
+  </si>
+  <si>
+    <t>Yap,Nicholas</t>
+  </si>
+  <si>
+    <t>14.5X30</t>
+  </si>
+  <si>
+    <t>Chaney,Jack</t>
+  </si>
+  <si>
+    <t>Chung,Hanna</t>
+  </si>
+  <si>
+    <t>Fujimoto,Andrew</t>
+  </si>
+  <si>
+    <t>Marino,Frank</t>
+  </si>
+  <si>
+    <t>Martini,Marco</t>
+  </si>
+  <si>
+    <t>Martins,Anket</t>
+  </si>
+  <si>
+    <t>McBride,Lindsey</t>
+  </si>
+  <si>
+    <t>Melton,Dawson</t>
+  </si>
+  <si>
+    <t>Rahman,Nadia</t>
+  </si>
+  <si>
+    <t>Randall,Conrad</t>
+  </si>
+  <si>
+    <t>Shegogue,Thomas</t>
+  </si>
+  <si>
+    <t>Stallone,Thomas</t>
+  </si>
+  <si>
+    <t>Viani,Jared</t>
+  </si>
+  <si>
+    <t>Zegunia,Julia</t>
+  </si>
+  <si>
+    <t>Annor,Reginald</t>
+  </si>
+  <si>
+    <t>Chilukuri,Sathya</t>
+  </si>
+  <si>
+    <t>Ettinger,Sophie</t>
+  </si>
+  <si>
+    <t>Fancher,Phillip</t>
+  </si>
+  <si>
+    <t>Hunt,Elyse</t>
+  </si>
+  <si>
+    <t>Isaac,Charles</t>
+  </si>
+  <si>
+    <t>Kim,Leo</t>
+  </si>
+  <si>
+    <t>Long,John</t>
+  </si>
+  <si>
+    <t>Perez,Rodrigo</t>
+  </si>
+  <si>
+    <t>Scalfani-Cohen,Andrew</t>
+  </si>
+  <si>
+    <t>Szymanski,Zoe</t>
+  </si>
+  <si>
+    <t>Teague,Katie</t>
+  </si>
+  <si>
+    <t>Tremel,Pulani</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -448,12 +448,6 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1244,138 +1238,138 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>5</v>
+        <v>41</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>6</v>
+        <v>42</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>7</v>
+        <v>43</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>8</v>
+        <v>44</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>14</v>
+        <v>50</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
       <c r="V1" s="5" t="s">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="X1" s="5" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="Y1" s="5" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="Z1" s="5" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="AA1" s="6" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E2" s="11">
         <v>0</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G2" s="11">
         <v>0</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I2" s="11">
         <v>0</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K2" s="11">
         <v>0</v>
       </c>
       <c r="L2" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M2" s="11">
         <v>0</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O2" s="11">
         <v>0</v>
       </c>
       <c r="P2" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q2" s="11">
         <v>0</v>
       </c>
       <c r="R2" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S2" s="11">
         <v>0</v>
       </c>
       <c r="T2" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U2" s="11">
         <v>0</v>
@@ -1401,64 +1395,64 @@
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E3" s="16">
         <v>0</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G3" s="16">
         <v>0</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I3" s="16">
         <v>0</v>
       </c>
       <c r="J3" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K3" s="16">
         <v>0</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M3" s="16">
         <v>0</v>
       </c>
       <c r="N3" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O3" s="16">
         <v>0</v>
       </c>
       <c r="P3" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q3" s="16">
         <v>0</v>
       </c>
       <c r="R3" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S3" s="16">
         <v>0</v>
       </c>
       <c r="T3" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U3" s="16">
         <v>0</v>
@@ -1484,64 +1478,64 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E4" s="11">
         <v>0</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G4" s="11">
         <v>0</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I4" s="11">
         <v>0</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K4" s="11">
         <v>0</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M4" s="11">
         <v>0</v>
       </c>
       <c r="N4" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O4" s="11">
         <v>0</v>
       </c>
       <c r="P4" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q4" s="11">
         <v>0</v>
       </c>
       <c r="R4" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S4" s="11">
         <v>0</v>
       </c>
       <c r="T4" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U4" s="11">
         <v>0</v>
@@ -1567,64 +1561,64 @@
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E5" s="16">
         <v>0</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G5" s="16">
         <v>0</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I5" s="16">
         <v>0</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K5" s="16">
         <v>0</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M5" s="16">
         <v>0</v>
       </c>
       <c r="N5" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O5" s="16">
         <v>0</v>
       </c>
       <c r="P5" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q5" s="16">
         <v>0</v>
       </c>
       <c r="R5" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S5" s="16">
         <v>0</v>
       </c>
       <c r="T5" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U5" s="16">
         <v>0</v>
@@ -1650,64 +1644,64 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E6" s="11">
         <v>0</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G6" s="11">
         <v>0</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I6" s="11">
         <v>0</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K6" s="11">
         <v>0</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M6" s="11">
         <v>0</v>
       </c>
       <c r="N6" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O6" s="11">
         <v>0</v>
       </c>
       <c r="P6" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q6" s="11">
         <v>0</v>
       </c>
       <c r="R6" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S6" s="11">
         <v>0</v>
       </c>
       <c r="T6" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U6" s="11">
         <v>0</v>
@@ -1733,64 +1727,64 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E7" s="16">
         <v>0</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G7" s="16">
         <v>0</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I7" s="16">
         <v>0</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K7" s="16">
         <v>0</v>
       </c>
       <c r="L7" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M7" s="16">
         <v>0</v>
       </c>
       <c r="N7" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O7" s="16">
         <v>0</v>
       </c>
       <c r="P7" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q7" s="16">
         <v>0</v>
       </c>
       <c r="R7" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S7" s="16">
         <v>0</v>
       </c>
       <c r="T7" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U7" s="16">
         <v>0</v>
@@ -1816,64 +1810,64 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>38</v>
+        <v>66</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E8" s="11">
         <v>0</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G8" s="11">
         <v>0</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I8" s="11">
         <v>0</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K8" s="11">
         <v>0</v>
       </c>
       <c r="L8" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M8" s="11">
         <v>0</v>
       </c>
       <c r="N8" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O8" s="11">
         <v>0</v>
       </c>
       <c r="P8" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q8" s="11">
         <v>0</v>
       </c>
       <c r="R8" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S8" s="11">
         <v>0</v>
       </c>
       <c r="T8" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U8" s="11">
         <v>0</v>
@@ -1899,64 +1893,64 @@
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E9" s="16">
         <v>0</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G9" s="16">
         <v>0</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I9" s="16">
         <v>0</v>
       </c>
       <c r="J9" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K9" s="16">
         <v>0</v>
       </c>
       <c r="L9" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M9" s="16">
         <v>0</v>
       </c>
       <c r="N9" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O9" s="16">
         <v>0</v>
       </c>
       <c r="P9" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q9" s="16">
         <v>0</v>
       </c>
       <c r="R9" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S9" s="16">
         <v>0</v>
       </c>
       <c r="T9" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U9" s="16">
         <v>0</v>
@@ -1982,64 +1976,64 @@
     </row>
     <row r="10" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="17" t="s">
-        <v>40</v>
+        <v>68</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E10" s="21">
         <v>0</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G10" s="21">
         <v>0</v>
       </c>
       <c r="H10" s="20" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I10" s="21">
         <v>0</v>
       </c>
       <c r="J10" s="20" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K10" s="21">
         <v>0</v>
       </c>
       <c r="L10" s="20" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M10" s="21">
         <v>0</v>
       </c>
       <c r="N10" s="20" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O10" s="21">
         <v>0</v>
       </c>
       <c r="P10" s="20" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q10" s="21">
         <v>0</v>
       </c>
       <c r="R10" s="20" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S10" s="21">
         <v>0</v>
       </c>
       <c r="T10" s="20" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U10" s="21">
         <v>0</v>
@@ -2065,64 +2059,64 @@
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>41</v>
+        <v>69</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D11" s="25" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E11" s="26">
         <v>0</v>
       </c>
       <c r="F11" s="25" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G11" s="26">
         <v>0</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I11" s="26">
         <v>0</v>
       </c>
       <c r="J11" s="25" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K11" s="26">
         <v>0</v>
       </c>
       <c r="L11" s="25" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M11" s="26">
         <v>0</v>
       </c>
       <c r="N11" s="25" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O11" s="26">
         <v>0</v>
       </c>
       <c r="P11" s="25" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q11" s="26">
         <v>0</v>
       </c>
       <c r="R11" s="25" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S11" s="26">
         <v>0</v>
       </c>
       <c r="T11" s="25" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U11" s="26">
         <v>0</v>
@@ -2148,64 +2142,64 @@
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E12" s="11">
         <v>0</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G12" s="11">
         <v>0</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I12" s="11">
         <v>0</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K12" s="11">
         <v>0</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M12" s="11">
         <v>0</v>
       </c>
       <c r="N12" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O12" s="11">
         <v>0</v>
       </c>
       <c r="P12" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q12" s="11">
         <v>0</v>
       </c>
       <c r="R12" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S12" s="11">
         <v>0</v>
       </c>
       <c r="T12" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U12" s="11">
         <v>0</v>
@@ -2231,64 +2225,64 @@
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A13" s="12" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E13" s="16">
         <v>0</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G13" s="16">
         <v>0</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I13" s="16">
         <v>0</v>
       </c>
       <c r="J13" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K13" s="16">
         <v>0</v>
       </c>
       <c r="L13" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M13" s="16">
         <v>0</v>
       </c>
       <c r="N13" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O13" s="16">
         <v>0</v>
       </c>
       <c r="P13" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q13" s="16">
         <v>0</v>
       </c>
       <c r="R13" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S13" s="16">
         <v>0</v>
       </c>
       <c r="T13" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U13" s="16">
         <v>0</v>
@@ -2314,64 +2308,64 @@
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E14" s="11">
         <v>0</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G14" s="11">
         <v>0</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I14" s="11">
         <v>0</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K14" s="11">
         <v>0</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M14" s="11">
         <v>0</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O14" s="11">
         <v>0</v>
       </c>
       <c r="P14" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q14" s="11">
         <v>0</v>
       </c>
       <c r="R14" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S14" s="11">
         <v>0</v>
       </c>
       <c r="T14" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U14" s="11">
         <v>0</v>
@@ -2397,64 +2391,64 @@
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E15" s="16">
         <v>0</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G15" s="16">
         <v>0</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I15" s="16">
         <v>0</v>
       </c>
       <c r="J15" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K15" s="16">
         <v>0</v>
       </c>
       <c r="L15" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M15" s="16">
         <v>0</v>
       </c>
       <c r="N15" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O15" s="16">
         <v>0</v>
       </c>
       <c r="P15" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q15" s="16">
         <v>0</v>
       </c>
       <c r="R15" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S15" s="16">
         <v>0</v>
       </c>
       <c r="T15" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U15" s="16">
         <v>0</v>
@@ -2480,64 +2474,64 @@
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E16" s="11">
         <v>0</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G16" s="11">
         <v>0</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I16" s="11">
         <v>0</v>
       </c>
       <c r="J16" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K16" s="11">
         <v>0</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M16" s="11">
         <v>0</v>
       </c>
       <c r="N16" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O16" s="11">
         <v>0</v>
       </c>
       <c r="P16" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q16" s="11">
         <v>0</v>
       </c>
       <c r="R16" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S16" s="11">
         <v>0</v>
       </c>
       <c r="T16" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U16" s="11">
         <v>0</v>
@@ -2563,64 +2557,64 @@
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A17" s="12" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>49</v>
+        <v>9</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E17" s="16">
         <v>0</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G17" s="16">
         <v>0</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I17" s="16">
         <v>0</v>
       </c>
       <c r="J17" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K17" s="16">
         <v>0</v>
       </c>
       <c r="L17" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M17" s="16">
         <v>0</v>
       </c>
       <c r="N17" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O17" s="16">
         <v>0</v>
       </c>
       <c r="P17" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q17" s="16">
         <v>0</v>
       </c>
       <c r="R17" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S17" s="16">
         <v>0</v>
       </c>
       <c r="T17" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U17" s="16">
         <v>0</v>
@@ -2646,64 +2640,64 @@
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E18" s="11">
         <v>0</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G18" s="11">
         <v>0</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I18" s="11">
         <v>0</v>
       </c>
       <c r="J18" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K18" s="11">
         <v>0</v>
       </c>
       <c r="L18" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M18" s="11">
         <v>0</v>
       </c>
       <c r="N18" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O18" s="11">
         <v>0</v>
       </c>
       <c r="P18" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q18" s="11">
         <v>0</v>
       </c>
       <c r="R18" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S18" s="11">
         <v>0</v>
       </c>
       <c r="T18" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U18" s="11">
         <v>0</v>
@@ -2729,64 +2723,64 @@
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E19" s="16">
         <v>0</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G19" s="16">
         <v>0</v>
       </c>
       <c r="H19" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I19" s="16">
         <v>0</v>
       </c>
       <c r="J19" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K19" s="16">
         <v>0</v>
       </c>
       <c r="L19" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M19" s="16">
         <v>0</v>
       </c>
       <c r="N19" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O19" s="16">
         <v>0</v>
       </c>
       <c r="P19" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q19" s="16">
         <v>0</v>
       </c>
       <c r="R19" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S19" s="16">
         <v>0</v>
       </c>
       <c r="T19" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U19" s="16">
         <v>0</v>
@@ -2812,64 +2806,64 @@
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
-        <v>53</v>
+        <v>78</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E20" s="11">
         <v>0</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G20" s="11">
         <v>0</v>
       </c>
       <c r="H20" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I20" s="11">
         <v>0</v>
       </c>
       <c r="J20" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K20" s="11">
         <v>0</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M20" s="11">
         <v>0</v>
       </c>
       <c r="N20" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O20" s="11">
         <v>0</v>
       </c>
       <c r="P20" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q20" s="11">
         <v>0</v>
       </c>
       <c r="R20" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S20" s="11">
         <v>0</v>
       </c>
       <c r="T20" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U20" s="11">
         <v>0</v>
@@ -2895,64 +2889,64 @@
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A21" s="12" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>49</v>
+        <v>9</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E21" s="16">
         <v>0</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G21" s="16">
         <v>0</v>
       </c>
       <c r="H21" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I21" s="16">
         <v>0</v>
       </c>
       <c r="J21" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K21" s="16">
         <v>0</v>
       </c>
       <c r="L21" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M21" s="16">
         <v>0</v>
       </c>
       <c r="N21" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O21" s="16">
         <v>0</v>
       </c>
       <c r="P21" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q21" s="16">
         <v>0</v>
       </c>
       <c r="R21" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S21" s="16">
         <v>0</v>
       </c>
       <c r="T21" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U21" s="16">
         <v>0</v>
@@ -2978,64 +2972,64 @@
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E22" s="11">
         <v>0</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G22" s="11">
         <v>0</v>
       </c>
       <c r="H22" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I22" s="11">
         <v>0</v>
       </c>
       <c r="J22" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K22" s="11">
         <v>0</v>
       </c>
       <c r="L22" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M22" s="11">
         <v>0</v>
       </c>
       <c r="N22" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O22" s="11">
         <v>0</v>
       </c>
       <c r="P22" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q22" s="11">
         <v>0</v>
       </c>
       <c r="R22" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S22" s="11">
         <v>0</v>
       </c>
       <c r="T22" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U22" s="11">
         <v>0</v>
@@ -3061,64 +3055,64 @@
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E23" s="16">
         <v>0</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G23" s="16">
         <v>0</v>
       </c>
       <c r="H23" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I23" s="16">
         <v>0</v>
       </c>
       <c r="J23" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K23" s="16">
         <v>0</v>
       </c>
       <c r="L23" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M23" s="16">
         <v>0</v>
       </c>
       <c r="N23" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O23" s="16">
         <v>0</v>
       </c>
       <c r="P23" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q23" s="16">
         <v>0</v>
       </c>
       <c r="R23" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S23" s="16">
         <v>0</v>
       </c>
       <c r="T23" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U23" s="16">
         <v>0</v>
@@ -3144,64 +3138,64 @@
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E24" s="11">
         <v>0</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G24" s="11">
         <v>0</v>
       </c>
       <c r="H24" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I24" s="11">
         <v>0</v>
       </c>
       <c r="J24" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K24" s="11">
         <v>0</v>
       </c>
       <c r="L24" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M24" s="11">
         <v>0</v>
       </c>
       <c r="N24" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O24" s="11">
         <v>0</v>
       </c>
       <c r="P24" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q24" s="11">
         <v>0</v>
       </c>
       <c r="R24" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S24" s="11">
         <v>0</v>
       </c>
       <c r="T24" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U24" s="11">
         <v>0</v>
@@ -3227,64 +3221,64 @@
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E25" s="16">
         <v>0</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G25" s="16">
         <v>0</v>
       </c>
       <c r="H25" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I25" s="16">
         <v>0</v>
       </c>
       <c r="J25" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K25" s="16">
         <v>0</v>
       </c>
       <c r="L25" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M25" s="16">
         <v>0</v>
       </c>
       <c r="N25" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O25" s="16">
         <v>0</v>
       </c>
       <c r="P25" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q25" s="16">
         <v>0</v>
       </c>
       <c r="R25" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S25" s="16">
         <v>0</v>
       </c>
       <c r="T25" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U25" s="16">
         <v>0</v>
@@ -3310,64 +3304,64 @@
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>49</v>
+        <v>9</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E26" s="11">
         <v>0</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G26" s="11">
         <v>0</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I26" s="11">
         <v>0</v>
       </c>
       <c r="J26" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K26" s="11">
         <v>0</v>
       </c>
       <c r="L26" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M26" s="11">
         <v>0</v>
       </c>
       <c r="N26" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O26" s="11">
         <v>0</v>
       </c>
       <c r="P26" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q26" s="11">
         <v>0</v>
       </c>
       <c r="R26" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S26" s="11">
         <v>0</v>
       </c>
       <c r="T26" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U26" s="11">
         <v>0</v>
@@ -3393,64 +3387,64 @@
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E27" s="16">
         <v>0</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G27" s="16">
         <v>0</v>
       </c>
       <c r="H27" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I27" s="16">
         <v>0</v>
       </c>
       <c r="J27" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K27" s="16">
         <v>0</v>
       </c>
       <c r="L27" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M27" s="16">
         <v>0</v>
       </c>
       <c r="N27" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O27" s="16">
         <v>0</v>
       </c>
       <c r="P27" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q27" s="16">
         <v>0</v>
       </c>
       <c r="R27" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S27" s="16">
         <v>0</v>
       </c>
       <c r="T27" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U27" s="16">
         <v>0</v>
@@ -3476,64 +3470,64 @@
     </row>
     <row r="28" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
-        <v>61</v>
+        <v>86</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E28" s="11">
         <v>0</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G28" s="11">
         <v>0</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I28" s="11">
         <v>0</v>
       </c>
       <c r="J28" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K28" s="11">
         <v>0</v>
       </c>
       <c r="L28" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M28" s="11">
         <v>0</v>
       </c>
       <c r="N28" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O28" s="11">
         <v>0</v>
       </c>
       <c r="P28" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q28" s="11">
         <v>0</v>
       </c>
       <c r="R28" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S28" s="11">
         <v>0</v>
       </c>
       <c r="T28" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U28" s="11">
         <v>0</v>
@@ -3559,64 +3553,64 @@
     </row>
     <row r="29" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A29" s="12" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E29" s="16">
         <v>0</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G29" s="16">
         <v>0</v>
       </c>
       <c r="H29" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I29" s="16">
         <v>0</v>
       </c>
       <c r="J29" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K29" s="16">
         <v>0</v>
       </c>
       <c r="L29" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="M29" s="16">
         <v>0</v>
       </c>
       <c r="N29" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="O29" s="16">
         <v>0</v>
       </c>
       <c r="P29" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q29" s="16">
         <v>0</v>
       </c>
       <c r="R29" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S29" s="16">
         <v>0</v>
       </c>
       <c r="T29" s="15" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U29" s="16">
         <v>0</v>
@@ -3642,13 +3636,13 @@
     </row>
     <row r="30" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="27" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D30" s="20">
         <v>16</v>
@@ -3657,19 +3651,19 @@
         <v>1</v>
       </c>
       <c r="F30" s="20" t="s">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="G30" s="21">
         <v>1</v>
       </c>
       <c r="H30" s="20" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="I30" s="21">
         <v>1</v>
       </c>
       <c r="J30" s="20" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K30" s="21">
         <v>0</v>
@@ -3681,25 +3675,25 @@
         <v>1</v>
       </c>
       <c r="N30" s="20" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="O30" s="21">
         <v>1</v>
       </c>
       <c r="P30" s="20" t="s">
-        <v>67</v>
+        <v>13</v>
       </c>
       <c r="Q30" s="21">
         <v>1</v>
       </c>
       <c r="R30" s="20" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S30" s="21">
         <v>0</v>
       </c>
       <c r="T30" s="20" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U30" s="21">
         <v>0</v>
@@ -3725,13 +3719,13 @@
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A31" s="22" t="s">
-        <v>68</v>
+        <v>90</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C31" s="24" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D31" s="25"/>
       <c r="E31" s="26"/>
@@ -3740,7 +3734,7 @@
       <c r="H31" s="25"/>
       <c r="I31" s="26"/>
       <c r="J31" s="25" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="K31" s="26">
         <v>0</v>
@@ -3754,13 +3748,13 @@
       <c r="R31" s="25"/>
       <c r="S31" s="26"/>
       <c r="T31" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U31" s="26">
         <v>0</v>
       </c>
       <c r="V31" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W31" s="31">
         <v>1</v>
@@ -3776,13 +3770,13 @@
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D32" s="10"/>
       <c r="E32" s="11"/>
@@ -3791,7 +3785,7 @@
       <c r="H32" s="10"/>
       <c r="I32" s="11"/>
       <c r="J32" s="10" t="s">
-        <v>71</v>
+        <v>15</v>
       </c>
       <c r="K32" s="11">
         <v>0</v>
@@ -3801,7 +3795,7 @@
         <v>1</v>
       </c>
       <c r="N32" s="10" t="s">
-        <v>72</v>
+        <v>16</v>
       </c>
       <c r="O32" s="11">
         <v>1</v>
@@ -3816,7 +3810,7 @@
         <v>1</v>
       </c>
       <c r="W32" s="33" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="X32" s="33"/>
       <c r="Y32" s="33"/>
@@ -3829,13 +3823,13 @@
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D33" s="15"/>
       <c r="E33" s="16"/>
@@ -3844,7 +3838,7 @@
       <c r="H33" s="15"/>
       <c r="I33" s="16"/>
       <c r="J33" s="15" t="s">
-        <v>74</v>
+        <v>17</v>
       </c>
       <c r="K33" s="16">
         <v>0</v>
@@ -3860,13 +3854,13 @@
       <c r="R33" s="15"/>
       <c r="S33" s="16"/>
       <c r="T33" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U33" s="16">
         <v>0</v>
       </c>
       <c r="V33" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W33" s="35">
         <v>1</v>
@@ -3882,13 +3876,13 @@
     </row>
     <row r="34" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D34" s="10"/>
       <c r="E34" s="11"/>
@@ -3897,7 +3891,7 @@
       <c r="H34" s="10"/>
       <c r="I34" s="11"/>
       <c r="J34" s="10" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="K34" s="11">
         <v>0</v>
@@ -3915,7 +3909,7 @@
       <c r="T34" s="10"/>
       <c r="U34" s="11"/>
       <c r="V34" s="33" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W34" s="33">
         <v>1</v>
@@ -3931,13 +3925,13 @@
     </row>
     <row r="35" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A35" s="12" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="16"/>
@@ -3946,7 +3940,7 @@
       <c r="H35" s="15"/>
       <c r="I35" s="16"/>
       <c r="J35" s="15" t="s">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="K35" s="16">
         <v>0</v>
@@ -3962,13 +3956,13 @@
       <c r="R35" s="15"/>
       <c r="S35" s="16"/>
       <c r="T35" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U35" s="16">
         <v>0</v>
       </c>
       <c r="V35" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W35" s="35">
         <v>1</v>
@@ -3984,13 +3978,13 @@
     </row>
     <row r="36" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D36" s="10"/>
       <c r="E36" s="11"/>
@@ -3999,7 +3993,7 @@
       <c r="H36" s="10"/>
       <c r="I36" s="11"/>
       <c r="J36" s="10" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="K36" s="11">
         <v>0</v>
@@ -4017,7 +4011,7 @@
       <c r="T36" s="10"/>
       <c r="U36" s="11"/>
       <c r="V36" s="33" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W36" s="33">
         <v>1</v>
@@ -4033,13 +4027,13 @@
     </row>
     <row r="37" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A37" s="12" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D37" s="15"/>
       <c r="E37" s="16"/>
@@ -4048,7 +4042,7 @@
       <c r="H37" s="15"/>
       <c r="I37" s="16"/>
       <c r="J37" s="15" t="s">
-        <v>80</v>
+        <v>19</v>
       </c>
       <c r="K37" s="16">
         <v>0</v>
@@ -4069,7 +4063,7 @@
         <v>1</v>
       </c>
       <c r="W37" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="X37" s="35"/>
       <c r="Y37" s="35"/>
@@ -4082,13 +4076,13 @@
     </row>
     <row r="38" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D38" s="10"/>
       <c r="E38" s="11"/>
@@ -4097,7 +4091,7 @@
       <c r="H38" s="10"/>
       <c r="I38" s="11"/>
       <c r="J38" s="10" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="K38" s="11">
         <v>0</v>
@@ -4115,7 +4109,7 @@
       <c r="T38" s="10"/>
       <c r="U38" s="11"/>
       <c r="V38" s="33" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W38" s="33">
         <v>1</v>
@@ -4131,13 +4125,13 @@
     </row>
     <row r="39" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A39" s="12" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D39" s="15"/>
       <c r="E39" s="16"/>
@@ -4146,7 +4140,7 @@
       <c r="H39" s="15"/>
       <c r="I39" s="16"/>
       <c r="J39" s="15" t="s">
-        <v>71</v>
+        <v>15</v>
       </c>
       <c r="K39" s="16">
         <v>0</v>
@@ -4156,7 +4150,7 @@
         <v>1</v>
       </c>
       <c r="N39" s="15" t="s">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="O39" s="16">
         <v>1</v>
@@ -4171,7 +4165,7 @@
         <v>1</v>
       </c>
       <c r="W39" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="X39" s="35"/>
       <c r="Y39" s="35"/>
@@ -4184,13 +4178,13 @@
     </row>
     <row r="40" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D40" s="10"/>
       <c r="E40" s="11"/>
@@ -4199,7 +4193,7 @@
       <c r="H40" s="10"/>
       <c r="I40" s="11"/>
       <c r="J40" s="10" t="s">
-        <v>85</v>
+        <v>21</v>
       </c>
       <c r="K40" s="11">
         <v>0</v>
@@ -4217,7 +4211,7 @@
       <c r="T40" s="10"/>
       <c r="U40" s="11"/>
       <c r="V40" s="33" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W40" s="33">
         <v>1</v>
@@ -4233,13 +4227,13 @@
     </row>
     <row r="41" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A41" s="12" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D41" s="15"/>
       <c r="E41" s="16"/>
@@ -4248,7 +4242,7 @@
       <c r="H41" s="15"/>
       <c r="I41" s="16"/>
       <c r="J41" s="15" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="K41" s="16">
         <v>0</v>
@@ -4264,13 +4258,13 @@
       <c r="R41" s="15"/>
       <c r="S41" s="16"/>
       <c r="T41" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U41" s="16">
         <v>0</v>
       </c>
       <c r="V41" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W41" s="35">
         <v>1</v>
@@ -4286,13 +4280,13 @@
     </row>
     <row r="42" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A42" s="7" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D42" s="10"/>
       <c r="E42" s="11"/>
@@ -4301,7 +4295,7 @@
       <c r="H42" s="10"/>
       <c r="I42" s="11"/>
       <c r="J42" s="10" t="s">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="K42" s="11">
         <v>0</v>
@@ -4319,7 +4313,7 @@
       <c r="T42" s="10"/>
       <c r="U42" s="11"/>
       <c r="V42" s="33" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W42" s="33">
         <v>1</v>
@@ -4335,13 +4329,13 @@
     </row>
     <row r="43" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A43" s="12" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D43" s="15"/>
       <c r="E43" s="16"/>
@@ -4350,13 +4344,13 @@
       <c r="H43" s="15"/>
       <c r="I43" s="16"/>
       <c r="J43" s="15" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="K43" s="16">
         <v>0</v>
       </c>
       <c r="L43" s="15" t="s">
-        <v>67</v>
+        <v>13</v>
       </c>
       <c r="M43" s="16">
         <v>1</v>
@@ -4368,13 +4362,13 @@
       <c r="R43" s="15"/>
       <c r="S43" s="16"/>
       <c r="T43" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U43" s="16">
         <v>0</v>
       </c>
       <c r="V43" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W43" s="35">
         <v>1</v>
@@ -4390,13 +4384,13 @@
     </row>
     <row r="44" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="27" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C44" s="19" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D44" s="20"/>
       <c r="E44" s="21"/>
@@ -4405,7 +4399,7 @@
       <c r="H44" s="20"/>
       <c r="I44" s="21"/>
       <c r="J44" s="20" t="s">
-        <v>90</v>
+        <v>22</v>
       </c>
       <c r="K44" s="21">
         <v>0</v>
@@ -4415,7 +4409,7 @@
         <v>1</v>
       </c>
       <c r="N44" s="20" t="s">
-        <v>91</v>
+        <v>23</v>
       </c>
       <c r="O44" s="21">
         <v>1</v>
@@ -4430,7 +4424,7 @@
         <v>1</v>
       </c>
       <c r="W44" s="33" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="X44" s="29"/>
       <c r="Y44" s="29"/>
@@ -4443,13 +4437,13 @@
     </row>
     <row r="45" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A45" s="22" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="C45" s="24" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D45" s="25"/>
       <c r="E45" s="26"/>
@@ -4458,7 +4452,7 @@
       <c r="H45" s="25"/>
       <c r="I45" s="26"/>
       <c r="J45" s="25" t="s">
-        <v>94</v>
+        <v>25</v>
       </c>
       <c r="K45" s="26">
         <v>1</v>
@@ -4470,7 +4464,7 @@
         <v>1</v>
       </c>
       <c r="N45" s="25" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="O45" s="26">
         <v>1</v>
@@ -4482,13 +4476,13 @@
         <v>0</v>
       </c>
       <c r="T45" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U45" s="26">
         <v>0</v>
       </c>
       <c r="V45" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W45" s="31">
         <v>1</v>
@@ -4504,13 +4498,13 @@
     </row>
     <row r="46" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A46" s="7" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D46" s="10"/>
       <c r="E46" s="11"/>
@@ -4519,7 +4513,7 @@
       <c r="H46" s="10"/>
       <c r="I46" s="11"/>
       <c r="J46" s="10" t="s">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="K46" s="11">
         <v>1</v>
@@ -4531,7 +4525,7 @@
         <v>1</v>
       </c>
       <c r="N46" s="10" t="s">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="O46" s="11">
         <v>1</v>
@@ -4539,17 +4533,17 @@
       <c r="P46" s="10"/>
       <c r="Q46" s="11"/>
       <c r="R46" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S46" s="11">
         <v>0</v>
       </c>
       <c r="T46" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U46" s="11"/>
       <c r="V46" s="33" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W46" s="33">
         <v>1</v>
@@ -4565,13 +4559,13 @@
     </row>
     <row r="47" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A47" s="12" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D47" s="15"/>
       <c r="E47" s="16"/>
@@ -4580,7 +4574,7 @@
       <c r="H47" s="15"/>
       <c r="I47" s="16"/>
       <c r="J47" s="15" t="s">
-        <v>97</v>
+        <v>26</v>
       </c>
       <c r="K47" s="16">
         <v>1</v>
@@ -4603,7 +4597,7 @@
         <v>1</v>
       </c>
       <c r="W47" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="X47" s="35"/>
       <c r="Y47" s="35"/>
@@ -4616,13 +4610,13 @@
     </row>
     <row r="48" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D48" s="10"/>
       <c r="E48" s="11"/>
@@ -4631,7 +4625,7 @@
       <c r="H48" s="10"/>
       <c r="I48" s="11"/>
       <c r="J48" s="10" t="s">
-        <v>67</v>
+        <v>13</v>
       </c>
       <c r="K48" s="11">
         <v>1</v>
@@ -4643,7 +4637,7 @@
         <v>1</v>
       </c>
       <c r="N48" s="10" t="s">
-        <v>67</v>
+        <v>13</v>
       </c>
       <c r="O48" s="11">
         <v>1</v>
@@ -4651,17 +4645,17 @@
       <c r="P48" s="10"/>
       <c r="Q48" s="11"/>
       <c r="R48" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S48" s="11">
         <v>0</v>
       </c>
       <c r="T48" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U48" s="11"/>
       <c r="V48" s="33" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W48" s="33">
         <v>1</v>
@@ -4677,13 +4671,13 @@
     </row>
     <row r="49" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A49" s="12" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D49" s="15"/>
       <c r="E49" s="16"/>
@@ -4692,7 +4686,7 @@
       <c r="H49" s="15"/>
       <c r="I49" s="16"/>
       <c r="J49" s="15" t="s">
-        <v>97</v>
+        <v>26</v>
       </c>
       <c r="K49" s="16">
         <v>1</v>
@@ -4715,7 +4709,7 @@
         <v>1</v>
       </c>
       <c r="W49" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="X49" s="35"/>
       <c r="Y49" s="35"/>
@@ -4728,13 +4722,13 @@
     </row>
     <row r="50" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A50" s="7" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D50" s="10"/>
       <c r="E50" s="11"/>
@@ -4743,7 +4737,7 @@
       <c r="H50" s="10"/>
       <c r="I50" s="11"/>
       <c r="J50" s="10" t="s">
-        <v>101</v>
+        <v>27</v>
       </c>
       <c r="K50" s="11">
         <v>1</v>
@@ -4759,17 +4753,17 @@
       <c r="P50" s="10"/>
       <c r="Q50" s="11"/>
       <c r="R50" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S50" s="11">
         <v>0</v>
       </c>
       <c r="T50" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U50" s="11"/>
       <c r="V50" s="33" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W50" s="33">
         <v>1</v>
@@ -4785,13 +4779,13 @@
     </row>
     <row r="51" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A51" s="12" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D51" s="15"/>
       <c r="E51" s="16"/>
@@ -4800,7 +4794,7 @@
       <c r="H51" s="15"/>
       <c r="I51" s="16"/>
       <c r="J51" s="15" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="K51" s="16">
         <v>1</v>
@@ -4820,13 +4814,13 @@
         <v>0</v>
       </c>
       <c r="T51" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U51" s="16">
         <v>0</v>
       </c>
       <c r="V51" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W51" s="35">
         <v>1</v>
@@ -4842,13 +4836,13 @@
     </row>
     <row r="52" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A52" s="7" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D52" s="10"/>
       <c r="E52" s="11"/>
@@ -4857,7 +4851,7 @@
       <c r="H52" s="10"/>
       <c r="I52" s="11"/>
       <c r="J52" s="10" t="s">
-        <v>104</v>
+        <v>28</v>
       </c>
       <c r="K52" s="11">
         <v>1</v>
@@ -4873,17 +4867,17 @@
       <c r="P52" s="10"/>
       <c r="Q52" s="11"/>
       <c r="R52" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S52" s="11">
         <v>0</v>
       </c>
       <c r="T52" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U52" s="11"/>
       <c r="V52" s="33" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W52" s="33">
         <v>1</v>
@@ -4899,13 +4893,13 @@
     </row>
     <row r="53" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A53" s="12" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D53" s="15"/>
       <c r="E53" s="16"/>
@@ -4914,7 +4908,7 @@
       <c r="H53" s="15"/>
       <c r="I53" s="16"/>
       <c r="J53" s="15" t="s">
-        <v>106</v>
+        <v>29</v>
       </c>
       <c r="K53" s="16">
         <v>1</v>
@@ -4926,13 +4920,13 @@
         <v>1</v>
       </c>
       <c r="N53" s="15" t="s">
-        <v>94</v>
+        <v>25</v>
       </c>
       <c r="O53" s="16">
         <v>1</v>
       </c>
       <c r="P53" s="15" t="s">
-        <v>107</v>
+        <v>30</v>
       </c>
       <c r="Q53" s="16">
         <v>1</v>
@@ -4942,13 +4936,13 @@
         <v>0</v>
       </c>
       <c r="T53" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U53" s="16">
         <v>0</v>
       </c>
       <c r="V53" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W53" s="35">
         <v>1</v>
@@ -4964,13 +4958,13 @@
     </row>
     <row r="54" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A54" s="7" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D54" s="10"/>
       <c r="E54" s="11"/>
@@ -4979,7 +4973,7 @@
       <c r="H54" s="10"/>
       <c r="I54" s="11"/>
       <c r="J54" s="10" t="s">
-        <v>109</v>
+        <v>31</v>
       </c>
       <c r="K54" s="11">
         <v>1</v>
@@ -4991,29 +4985,29 @@
         <v>1</v>
       </c>
       <c r="N54" s="10" t="s">
-        <v>110</v>
+        <v>32</v>
       </c>
       <c r="O54" s="11">
         <v>1</v>
       </c>
       <c r="P54" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Q54" s="11">
         <v>0</v>
       </c>
       <c r="R54" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="S54" s="11">
         <v>0</v>
       </c>
       <c r="T54" s="10" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="U54" s="11"/>
       <c r="V54" s="33" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W54" s="33">
         <v>1</v>
@@ -5029,13 +5023,13 @@
     </row>
     <row r="55" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A55" s="12" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D55" s="15"/>
       <c r="E55" s="16"/>
@@ -5044,7 +5038,7 @@
       <c r="H55" s="15"/>
       <c r="I55" s="16"/>
       <c r="J55" s="15" t="s">
-        <v>80</v>
+        <v>19</v>
       </c>
       <c r="K55" s="16">
         <v>1</v>
@@ -5065,7 +5059,7 @@
         <v>1</v>
       </c>
       <c r="W55" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="X55" s="35"/>
       <c r="Y55" s="35"/>
@@ -5078,13 +5072,13 @@
     </row>
     <row r="56" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A56" s="7" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D56" s="10"/>
       <c r="E56" s="11"/>
@@ -5093,7 +5087,7 @@
       <c r="H56" s="10"/>
       <c r="I56" s="11"/>
       <c r="J56" s="10" t="s">
-        <v>97</v>
+        <v>26</v>
       </c>
       <c r="K56" s="11">
         <v>1</v>
@@ -5114,7 +5108,7 @@
         <v>1</v>
       </c>
       <c r="W56" s="33" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="X56" s="33"/>
       <c r="Y56" s="33"/>
@@ -5127,13 +5121,13 @@
     </row>
     <row r="57" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="39" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B57" s="40" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="C57" s="41" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D57" s="42"/>
       <c r="E57" s="43"/>
@@ -5142,7 +5136,7 @@
       <c r="H57" s="42"/>
       <c r="I57" s="43"/>
       <c r="J57" s="42" t="s">
-        <v>114</v>
+        <v>33</v>
       </c>
       <c r="K57" s="43">
         <v>1</v>
@@ -5163,7 +5157,7 @@
         <v>1</v>
       </c>
       <c r="W57" s="31" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="X57" s="44"/>
       <c r="Y57" s="44"/>
@@ -5179,11 +5173,11 @@
     </row>
     <row r="59" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="48" t="s">
-        <v>115</v>
+        <v>34</v>
       </c>
       <c r="B59" s="49"/>
       <c r="C59" s="48" t="s">
-        <v>116</v>
+        <v>35</v>
       </c>
     </row>
     <row r="60" spans="1:27" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Adding subamdin account, changing background image interface
</commit_message>
<xml_diff>
--- a/cadet_data/CadetData_Blues.xlsx
+++ b/cadet_data/CadetData_Blues.xlsx
@@ -574,8 +574,10 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>0</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -681,8 +683,10 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>0</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1109,8 +1113,10 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>0</v>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Adding filelocks to ensure that simultaneous edits do not overritw each other
</commit_message>
<xml_diff>
--- a/cadet_data/CadetData_Blues.xlsx
+++ b/cadet_data/CadetData_Blues.xlsx
@@ -685,7 +685,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -792,8 +792,10 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>0</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1110,12 +1112,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">

</xml_diff>